<commit_message>
Order page updates: Friday fulfillment, friendly pricing, Pantry Box flavor picker
- Change fulfillment day Saturday -> Friday everywhere (order page, confirmation
  email, launch graphic, bake log, docs) — Jaime isn't delivering Saturdays.
- Switch to friendly launch pricing (classic loaf $9, specialty $12, muffins $12,
  cookies $15, jam $8, Pantry Box $26).
- Rename the Cookies menu banner to "Sourdough Cookies".
- Pantry Box now shows loaf/jam/cookie dropdowns (appear only when a box is added)
  populated from the current menu, so weekly flavor changes need no box edits. The
  chosen flavors flow into the order summary and both emails.
- Regenerate launch-graphic.png and bake-log.xlsx.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/marketing/bake-log.xlsx
+++ b/marketing/bake-log.xlsx
@@ -138,7 +138,7 @@
     <t>Bake for pickup date →</t>
   </si>
   <si>
-    <t>(type any Saturday here — the numbers below update)</t>
+    <t>(type any Friday here — the numbers below update)</t>
   </si>
   <si>
     <t>PRODUCT</t>
@@ -174,7 +174,7 @@
     <t>What this is</t>
   </si>
   <si>
-    <t>A running log of every bread-drop order, plus an automatic "what to bake" list for each Saturday.</t>
+    <t>A running log of every bread-drop order, plus an automatic "what to bake" list for each Friday.</t>
   </si>
   <si>
     <t>Each week</t>
@@ -183,13 +183,13 @@
     <t>1. As orders arrive, add a row on the ORDERS tab. Each order emails you the details — copy them in.</t>
   </si>
   <si>
-    <t>2. Put the Saturday pickup date in the "Pickup Date" column for every order in that drop.</t>
+    <t>2. Put the Friday pickup date in the "Pickup Date" column for every order in that drop.</t>
   </si>
   <si>
     <t>3. When a Venmo/Zelle payment lands, set that order’s "Paid?" to Yes (unpaid rows glow clay-orange).</t>
   </si>
   <si>
-    <t>4. On the WEEKLY BAKE LIST tab, type that Saturday’s date in the highlighted box.</t>
+    <t>4. On the WEEKLY BAKE LIST tab, type that Friday’s date in the highlighted box.</t>
   </si>
   <si>
     <t xml:space="preserve">   The tab instantly shows how many of each item to bake, revenue, pickups vs. deliveries, and who still owes.</t>
@@ -920,7 +920,7 @@
     </row>
     <row r="3" ht="18" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
-        <v>46242.20833333333</v>
+        <v>46241.20833333333</v>
       </c>
       <c r="B3" s="4">
         <v>46238.59166666667</v>
@@ -971,7 +971,7 @@
     </row>
     <row r="4" ht="18" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
-        <v>46242.20833333333</v>
+        <v>46241.20833333333</v>
       </c>
       <c r="B4" s="4">
         <v>46238.59166666667</v>
@@ -1024,7 +1024,7 @@
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
-        <v>46242.20833333333</v>
+        <v>46241.20833333333</v>
       </c>
       <c r="B5" s="4">
         <v>46238.59166666667</v>
@@ -10256,7 +10256,7 @@
         <v>40</v>
       </c>
       <c r="B3" s="11">
-        <v>46242.20833333333</v>
+        <v>46241.20833333333</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>